<commit_message>
adding cotton and barley prices data to the dataset
</commit_message>
<xml_diff>
--- a/data/raw/data.xlsx
+++ b/data/raw/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Economics-B1\Desktop\syrian-wheat-supply-response-model\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A68545-BC91-4104-9975-3D2B6603DB4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE34CF5F-BEBC-4317-8A2D-F5FC72346BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9915" yWindow="1200" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -34,30 +34,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Production (Ton)</t>
-  </si>
-  <si>
-    <t>Area (Hectar)</t>
-  </si>
-  <si>
-    <t>Yeild (Ton/Ha)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Inflation (GDP Deflator)</t>
-  </si>
-  <si>
-    <t>Price Per Ton (Syrian Lira)</t>
   </si>
   <si>
     <t>Agriculture Stress Index (VHI % below 35)</t>
   </si>
   <si>
     <t>Political Stability (0 to 100)</t>
+  </si>
+  <si>
+    <t>Production (tons)</t>
+  </si>
+  <si>
+    <t>Area (Hectars)</t>
+  </si>
+  <si>
+    <t>Yeild (tons/Hectar)</t>
+  </si>
+  <si>
+    <t>Year+A:H</t>
+  </si>
+  <si>
+    <t>Wheat Price (Syrian Lira per ton)</t>
+  </si>
+  <si>
+    <t>Barley Price (Syrian Lira per ton)</t>
+  </si>
+  <si>
+    <t>Cotton Price (Syrian Lira per ton)</t>
   </si>
 </sst>
 </file>
@@ -103,7 +109,6 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -116,6 +121,9 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -398,675 +406,760 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="22.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>2002</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>4775442</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>1679350</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>2.8439999999999999</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="5">
         <v>11300</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <v>6.1699999999999998E-2</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="3">
         <v>100.94576420473101</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="3">
         <v>67.084905699999993</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+      <c r="I2" s="6">
+        <v>30750</v>
+      </c>
+      <c r="J2" s="6">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>2003</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>4912993</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>1796015</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>2.7349999999999999</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="5">
         <v>11300</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <v>4.0999999999999995E-3</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>105.443556501415</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <v>65.4226934</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="I3" s="6">
+        <v>30750</v>
+      </c>
+      <c r="J3" s="6">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>2004</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>4537459</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>1831226</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>2.4780000000000002</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>11300</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>1.9299999999999998E-2</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>116.332327608065</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="3">
         <v>59.428158599999996</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+      <c r="I4" s="6">
+        <v>30750</v>
+      </c>
+      <c r="J4" s="6">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>2005</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>4668746</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>1903826</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>2.452</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="5">
         <v>11300</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>1.06E-2</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="3">
         <v>130.23412142817</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="3">
         <v>57.969138799999996</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+      <c r="I5" s="6">
+        <v>30750</v>
+      </c>
+      <c r="J5" s="6">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>2006</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>4931525</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>1786659</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>2.76</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="5">
         <v>11300</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="4">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>142.081376634202</v>
       </c>
-      <c r="H6" s="4">
+      <c r="H6" s="3">
         <v>56.797991799999998</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+      <c r="I6" s="6">
+        <v>30750</v>
+      </c>
+      <c r="J6" s="6">
+        <v>9500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
         <v>2007</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>4041100</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="2">
         <v>1667732</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="2">
         <v>2.423</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="5">
         <v>11300</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="4">
         <v>0.13800000000000001</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="3">
         <v>157.381930229012</v>
       </c>
-      <c r="H7" s="4">
+      <c r="H7" s="3">
         <v>56.274659399999997</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+      <c r="I7" s="6">
+        <v>41000</v>
+      </c>
+      <c r="J7" s="6">
+        <v>9500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
         <v>2008</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>2139313</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="2">
         <v>1485991</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="2">
         <v>1.44</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="5">
         <v>16750</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="4">
         <v>0.56059999999999999</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="3">
         <v>182.484578193158</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="3">
         <v>55.733806399999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+      <c r="I8" s="6">
+        <v>42000</v>
+      </c>
+      <c r="J8" s="6">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
         <v>2009</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>3701784</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="2">
         <v>1437375</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="2">
         <v>2.5750000000000002</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="5">
         <v>19750</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="4">
         <v>6.7199999999999996E-2</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="3">
         <v>177.41063086382499</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="3">
         <v>56.900823099999997</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
+      <c r="I9" s="6">
+        <v>42000</v>
+      </c>
+      <c r="J9" s="6">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
         <v>2010</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>3083082</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
         <v>1599108</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>1.9279999999999999</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="5">
         <v>20250</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="4">
         <v>3.0499999999999999E-2</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10" s="3">
         <v>189.65143431420799</v>
       </c>
-      <c r="H10" s="4">
+      <c r="H10" s="3">
         <v>46.805809099999998</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
+      <c r="I10" s="6">
+        <v>42000</v>
+      </c>
+      <c r="J10" s="6">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
         <v>2011</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>3858331</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="2">
         <v>1521038</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="2">
         <v>2.5369999999999999</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="5">
         <v>21250</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="4">
         <v>0.14960000000000001</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="3">
         <v>211.60139950226301</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <v>29.446354199999998</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
+      <c r="I11" s="6">
+        <v>51000</v>
+      </c>
+      <c r="J11" s="6">
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
         <v>2012</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <v>3609096</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="2">
         <v>1602814</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>2.2519999999999998</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="5">
         <v>22250</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="4">
         <v>8.1600000000000006E-2</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>267.13841396733397</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="3">
         <v>23.951639</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+      <c r="I12" s="6">
+        <v>100000</v>
+      </c>
+      <c r="J12" s="6">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
         <v>2013</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <v>3182111</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="2">
         <v>1374077</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>2.3159999999999998</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="5">
         <v>36500</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="4">
         <v>4.8099999999999997E-2</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="3">
         <v>352.009618472537</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="3">
         <v>23.771323899999999</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+      <c r="I13" s="6">
+        <v>110000</v>
+      </c>
+      <c r="J13" s="6">
+        <v>31000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
         <v>2014</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <v>2024332</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <v>1287885</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="2">
         <v>1.5720000000000001</v>
       </c>
-      <c r="E14" s="6">
+      <c r="E14" s="5">
         <v>44500</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="4">
         <v>0.46610000000000001</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="3">
         <v>482.58612920502202</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="3">
         <v>25.7574443</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+      <c r="I14" s="6">
+        <v>110000</v>
+      </c>
+      <c r="J14" s="6">
+        <v>33000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
         <v>2015</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="2">
         <v>2861628</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="2">
         <v>1197200</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <v>2.39</v>
       </c>
-      <c r="E15" s="6">
+      <c r="E15" s="5">
         <v>61000</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="4">
         <v>2.5499999999999998E-2</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="3">
         <v>667.00347475630599</v>
       </c>
-      <c r="H15" s="4">
+      <c r="H15" s="3">
         <v>24.245802899999997</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+      <c r="I15" s="6">
+        <v>140000</v>
+      </c>
+      <c r="J15" s="6">
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
         <v>2016</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="2">
         <v>1726247</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="2">
         <v>1178506</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="2">
         <v>1.4650000000000001</v>
       </c>
-      <c r="E16" s="6">
+      <c r="E16" s="5">
         <v>100000</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="4">
         <v>0.43340000000000001</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="3">
         <v>912.93555832872596</v>
       </c>
-      <c r="H16" s="4">
+      <c r="H16" s="3">
         <v>21.5585068</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
+      <c r="I16" s="6">
+        <v>235000</v>
+      </c>
+      <c r="J16" s="6">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
         <v>2017</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="2">
         <v>1850740</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="2">
         <v>1169911</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="2">
         <v>1.5820000000000001</v>
       </c>
-      <c r="E17" s="6">
+      <c r="E17" s="5">
         <v>140000</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="4">
         <v>0.2336</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17" s="3">
         <v>1252.7395831561801</v>
       </c>
-      <c r="H17" s="4">
+      <c r="H17" s="3">
         <v>24.123397900000001</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
+      <c r="I17" s="6">
+        <v>300000</v>
+      </c>
+      <c r="J17" s="6">
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
         <v>2018</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="2">
         <v>1222988</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="2">
         <v>1096818</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="2">
         <v>1.115</v>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="5">
         <v>175000</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="4">
         <v>0.56289999999999996</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="3">
         <v>1417.94914744364</v>
       </c>
-      <c r="H18" s="4">
+      <c r="H18" s="3">
         <v>24.4910213</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="3">
+      <c r="I18" s="6">
+        <v>350000</v>
+      </c>
+      <c r="J18" s="6">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
         <v>2019</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19" s="2">
         <v>3085097</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="2">
         <v>1345607</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="2">
         <v>2.2930000000000001</v>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="5">
         <v>185000</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="4">
         <v>7.0999999999999995E-3</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19" s="3">
         <v>1699.1476824066201</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="3">
         <v>23.998244399999997</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
+      <c r="I19" s="6">
+        <v>360000</v>
+      </c>
+      <c r="J19" s="6">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
         <v>2020</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20" s="2">
         <v>2848472</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="2">
         <v>1350538</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="2">
         <v>2.109</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="5">
         <v>400000</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="4">
         <v>4.1799999999999997E-2</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20" s="3">
         <v>2802.37597291058</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="3">
         <v>25.689845599999998</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
+      <c r="I20" s="6">
+        <v>700000</v>
+      </c>
+      <c r="J20" s="6">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
         <v>2021</v>
       </c>
-      <c r="B21" s="3">
+      <c r="B21" s="2">
         <v>1951806</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="2">
         <v>1567262</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="2">
         <v>1.2450000000000001</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="5">
         <v>900000</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="4">
         <v>0.30570000000000003</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21" s="3">
         <v>6120.3674956709601</v>
       </c>
-      <c r="H21" s="4">
+      <c r="H21" s="3">
         <v>25.333728399999998</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
+      <c r="I21" s="6">
+        <v>2500000</v>
+      </c>
+      <c r="J21" s="6">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
         <v>2022</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B22" s="2">
         <v>1551605</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C22" s="2">
         <v>1184237</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="2">
         <v>1.31</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="5">
         <v>2000000</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="4">
         <v>0.38420000000000004</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22" s="3">
         <v>12692.121336549801</v>
       </c>
-      <c r="H22" s="4">
+      <c r="H22" s="3">
         <v>24.245223899999999</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="3">
+      <c r="I22" s="6">
+        <v>4000000</v>
+      </c>
+      <c r="J22" s="6">
+        <v>1800000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
         <v>2023</v>
       </c>
-      <c r="B23" s="3">
+      <c r="B23" s="2">
         <v>3080351</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C23" s="2">
         <v>1335667</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="2">
         <v>2.306</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="5">
         <v>2800000</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="4">
         <v>9.0500000000000011E-2</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23" s="3">
         <f xml:space="preserve"> G22*1.93</f>
         <v>24495.794179541113</v>
       </c>
-      <c r="H23" s="4">
+      <c r="H23" s="3">
         <v>24.2511221</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
-        <v>2024</v>
-      </c>
-      <c r="B24" s="3">
-        <v>2400000</v>
-      </c>
-      <c r="C24" s="3">
-        <v>1270000</v>
-      </c>
-      <c r="D24" s="3">
-        <v>1.889</v>
-      </c>
-      <c r="E24" s="6">
-        <v>5500000</v>
-      </c>
-      <c r="F24" s="5">
-        <v>3.9100000000000003E-2</v>
-      </c>
-      <c r="G24" s="4">
-        <f>G23*1.721</f>
-        <v>42157.261782990259</v>
-      </c>
-      <c r="H24" s="4">
-        <v>25.44</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="3">
-        <v>2025</v>
-      </c>
-      <c r="B25" s="3">
-        <v>900000</v>
-      </c>
-      <c r="C25" s="3">
-        <v>1100000</v>
-      </c>
-      <c r="D25" s="3">
-        <v>0.81799999999999995</v>
-      </c>
-      <c r="E25" s="6">
-        <v>4600000</v>
-      </c>
-      <c r="F25" s="5">
-        <v>0.76139999999999997</v>
-      </c>
-      <c r="G25" s="4">
-        <f>G24*1.115</f>
-        <v>47005.346888034139</v>
-      </c>
-      <c r="H25" s="4">
-        <v>25.44</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F30" s="1"/>
+      <c r="I23" s="6">
+        <v>10000000</v>
+      </c>
+      <c r="J23" s="6">
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F30"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update data import and processing for revised dataset
</commit_message>
<xml_diff>
--- a/data/raw/data.xlsx
+++ b/data/raw/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Economics-B1\Desktop\syrian-wheat-supply-response-model\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F09459C3-9021-49B1-A1D6-A3A7C0CC0821}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F92D07-5483-4B59-AB2B-69E3C34515E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1740" yWindow="2235" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" r:id="rId1"/>
@@ -34,15 +34,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Inflation (GDP Deflator)</t>
   </si>
   <si>
     <t>Agriculture Stress Index (VHI % below 35)</t>
-  </si>
-  <si>
-    <t>Political Stability (0 to 100)</t>
   </si>
   <si>
     <t>Production (tons)</t>
@@ -64,6 +61,12 @@
   </si>
   <si>
     <t>Year</t>
+  </si>
+  <si>
+    <t>Political Stability Index (0 to 100)</t>
+  </si>
+  <si>
+    <t>Government Effectiveness Index (1 to 100)</t>
   </si>
 </sst>
 </file>
@@ -111,19 +114,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -406,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -416,749 +419,819 @@
     <col min="5" max="5" width="31.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="38.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="30.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="39.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
         <v>2002</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>4775442</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>1679350</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>2.8439999999999999</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="6">
         <v>11300</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="5">
         <v>6.1699999999999998E-2</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="4">
         <v>100.94576420473101</v>
       </c>
       <c r="H2" s="3">
+        <v>26.8796836</v>
+      </c>
+      <c r="I2" s="4">
         <v>67.084905699999993</v>
       </c>
-      <c r="I2" s="6">
+      <c r="J2" s="2">
         <v>30750</v>
       </c>
-      <c r="J2" s="6">
+      <c r="K2" s="2">
         <v>12000</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
         <v>2003</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>4912993</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>1796015</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>2.7349999999999999</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="6">
         <v>11300</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="5">
         <v>4.0999999999999995E-3</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="4">
         <v>105.443556501415</v>
       </c>
       <c r="H3" s="3">
+        <v>22.864298999999999</v>
+      </c>
+      <c r="I3" s="4">
         <v>65.4226934</v>
       </c>
-      <c r="I3" s="6">
+      <c r="J3" s="2">
         <v>30750</v>
       </c>
-      <c r="J3" s="6">
+      <c r="K3" s="2">
         <v>7500</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
         <v>2004</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>4537459</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>1831226</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>2.4780000000000002</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>11300</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="5">
         <v>1.9299999999999998E-2</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="4">
         <v>116.332327608065</v>
       </c>
       <c r="H4" s="3">
+        <v>27.357922799999997</v>
+      </c>
+      <c r="I4" s="4">
         <v>59.428158599999996</v>
       </c>
-      <c r="I4" s="6">
+      <c r="J4" s="2">
         <v>30750</v>
       </c>
-      <c r="J4" s="6">
+      <c r="K4" s="2">
         <v>7500</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
         <v>2005</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="3">
         <v>4668746</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="3">
         <v>1903826</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>2.452</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="6">
         <v>11300</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="5">
         <v>1.06E-2</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="4">
         <v>130.23412142817</v>
       </c>
       <c r="H5" s="3">
+        <v>26.498462199999999</v>
+      </c>
+      <c r="I5" s="4">
         <v>57.969138799999996</v>
       </c>
-      <c r="I5" s="6">
+      <c r="J5" s="2">
         <v>30750</v>
       </c>
-      <c r="J5" s="6">
+      <c r="K5" s="2">
         <v>7500</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
         <v>2006</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="3">
         <v>4931525</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <v>1786659</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="3">
         <v>2.76</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="6">
         <v>11300</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="5">
         <v>6.4500000000000002E-2</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="4">
         <v>142.081376634202</v>
       </c>
       <c r="H6" s="3">
+        <v>31.462942399999999</v>
+      </c>
+      <c r="I6" s="4">
         <v>56.797991799999998</v>
       </c>
-      <c r="I6" s="6">
+      <c r="J6" s="2">
         <v>30750</v>
       </c>
-      <c r="J6" s="6">
+      <c r="K6" s="2">
         <v>9500</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
         <v>2007</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <v>4041100</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>1667732</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="3">
         <v>2.423</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="6">
         <v>11300</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="5">
         <v>0.13800000000000001</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="4">
         <v>157.381930229012</v>
       </c>
       <c r="H7" s="3">
+        <v>32.681981299999997</v>
+      </c>
+      <c r="I7" s="4">
         <v>56.274659399999997</v>
       </c>
-      <c r="I7" s="6">
+      <c r="J7" s="2">
         <v>41000</v>
       </c>
-      <c r="J7" s="6">
+      <c r="K7" s="2">
         <v>9500</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
         <v>2008</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <v>2139313</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
         <v>1485991</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="3">
         <v>1.44</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="6">
         <v>16750</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="5">
         <v>0.56059999999999999</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="4">
         <v>182.484578193158</v>
       </c>
       <c r="H8" s="3">
+        <v>36.2838694</v>
+      </c>
+      <c r="I8" s="4">
         <v>55.733806399999999</v>
       </c>
-      <c r="I8" s="6">
+      <c r="J8" s="2">
         <v>42000</v>
       </c>
-      <c r="J8" s="6">
+      <c r="K8" s="2">
         <v>15000</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <v>2009</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="3">
         <v>3701784</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="3">
         <v>1437375</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="3">
         <v>2.5750000000000002</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="6">
         <v>19750</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9" s="5">
         <v>6.7199999999999996E-2</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="4">
         <v>177.41063086382499</v>
       </c>
       <c r="H9" s="3">
+        <v>37.442940999999998</v>
+      </c>
+      <c r="I9" s="4">
         <v>56.900823099999997</v>
       </c>
-      <c r="I9" s="6">
+      <c r="J9" s="2">
         <v>42000</v>
       </c>
-      <c r="J9" s="6">
+      <c r="K9" s="2">
         <v>16000</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
         <v>2010</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="3">
         <v>3083082</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <v>1599108</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="3">
         <v>1.9279999999999999</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="6">
         <v>20250</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F10" s="5">
         <v>3.0499999999999999E-2</v>
       </c>
-      <c r="G10" s="3">
+      <c r="G10" s="4">
         <v>189.65143431420799</v>
       </c>
       <c r="H10" s="3">
+        <v>37.843196200000001</v>
+      </c>
+      <c r="I10" s="4">
         <v>46.805809099999998</v>
       </c>
-      <c r="I10" s="6">
+      <c r="J10" s="2">
         <v>42000</v>
       </c>
-      <c r="J10" s="6">
+      <c r="K10" s="2">
         <v>16000</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
         <v>2011</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="3">
         <v>3858331</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="3">
         <v>1521038</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="3">
         <v>2.5369999999999999</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="6">
         <v>21250</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F11" s="5">
         <v>0.14960000000000001</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="4">
         <v>211.60139950226301</v>
       </c>
       <c r="H11" s="3">
+        <v>37.943951200000001</v>
+      </c>
+      <c r="I11" s="4">
         <v>29.446354199999998</v>
       </c>
-      <c r="I11" s="6">
+      <c r="J11" s="2">
         <v>51000</v>
       </c>
-      <c r="J11" s="6">
+      <c r="K11" s="2">
         <v>17000</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
         <v>2012</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="3">
         <v>3609096</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="3">
         <v>1602814</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="3">
         <v>2.2519999999999998</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="6">
         <v>22250</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="5">
         <v>8.1600000000000006E-2</v>
       </c>
-      <c r="G12" s="3">
+      <c r="G12" s="4">
         <v>267.13841396733397</v>
       </c>
       <c r="H12" s="3">
+        <v>33.299698399999997</v>
+      </c>
+      <c r="I12" s="4">
         <v>23.951639</v>
       </c>
-      <c r="I12" s="6">
+      <c r="J12" s="2">
         <v>100000</v>
       </c>
-      <c r="J12" s="6">
+      <c r="K12" s="2">
         <v>20000</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <v>2013</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="3">
         <v>3182111</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="3">
         <v>1374077</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="3">
         <v>2.3159999999999998</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="6">
         <v>36500</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F13" s="5">
         <v>4.8099999999999997E-2</v>
       </c>
-      <c r="G13" s="3">
+      <c r="G13" s="4">
         <v>352.009618472537</v>
       </c>
       <c r="H13" s="3">
+        <v>29.264556799999998</v>
+      </c>
+      <c r="I13" s="4">
         <v>23.771323899999999</v>
       </c>
-      <c r="I13" s="6">
+      <c r="J13" s="2">
         <v>110000</v>
       </c>
-      <c r="J13" s="6">
+      <c r="K13" s="2">
         <v>31000</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
         <v>2014</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="3">
         <v>2024332</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="3">
         <v>1287885</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="3">
         <v>1.5720000000000001</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="6">
         <v>44500</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="5">
         <v>0.46610000000000001</v>
       </c>
-      <c r="G14" s="3">
+      <c r="G14" s="4">
         <v>482.58612920502202</v>
       </c>
       <c r="H14" s="3">
+        <v>31.578535199999997</v>
+      </c>
+      <c r="I14" s="4">
         <v>25.7574443</v>
       </c>
-      <c r="I14" s="6">
+      <c r="J14" s="2">
         <v>110000</v>
       </c>
-      <c r="J14" s="6">
+      <c r="K14" s="2">
         <v>33000</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
         <v>2015</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="3">
         <v>2861628</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="3">
         <v>1197200</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="3">
         <v>2.39</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="6">
         <v>61000</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F15" s="5">
         <v>2.5499999999999998E-2</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="4">
         <v>667.00347475630599</v>
       </c>
       <c r="H15" s="3">
+        <v>27.115967299999998</v>
+      </c>
+      <c r="I15" s="4">
         <v>24.245802899999997</v>
       </c>
-      <c r="I15" s="6">
+      <c r="J15" s="2">
         <v>140000</v>
       </c>
-      <c r="J15" s="6">
+      <c r="K15" s="2">
         <v>48000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
         <v>2016</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="3">
         <v>1726247</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="3">
         <v>1178506</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="3">
         <v>1.4650000000000001</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="6">
         <v>100000</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="5">
         <v>0.43340000000000001</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="4">
         <v>912.93555832872596</v>
       </c>
       <c r="H16" s="3">
+        <v>22.739003699999998</v>
+      </c>
+      <c r="I16" s="4">
         <v>21.5585068</v>
       </c>
-      <c r="I16" s="6">
+      <c r="J16" s="2">
         <v>235000</v>
       </c>
-      <c r="J16" s="6">
+      <c r="K16" s="2">
         <v>75000</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
         <v>2017</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="3">
         <v>1850740</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17" s="3">
         <v>1169911</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="3">
         <v>1.5820000000000001</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="6">
         <v>140000</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="5">
         <v>0.2336</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" s="4">
         <v>1252.7395831561801</v>
       </c>
       <c r="H17" s="3">
+        <v>22.741123099999999</v>
+      </c>
+      <c r="I17" s="4">
         <v>24.123397900000001</v>
       </c>
-      <c r="I17" s="6">
+      <c r="J17" s="2">
         <v>300000</v>
       </c>
-      <c r="J17" s="6">
+      <c r="K17" s="2">
         <v>110000</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
         <v>2018</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="3">
         <v>1222988</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="3">
         <v>1096818</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="3">
         <v>1.115</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="6">
         <v>175000</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="5">
         <v>0.56289999999999996</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="4">
         <v>1417.94914744364</v>
       </c>
       <c r="H18" s="3">
+        <v>22.752756399999999</v>
+      </c>
+      <c r="I18" s="4">
         <v>24.4910213</v>
       </c>
-      <c r="I18" s="6">
+      <c r="J18" s="2">
         <v>350000</v>
       </c>
-      <c r="J18" s="6">
+      <c r="K18" s="2">
         <v>130000</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="3">
         <v>2019</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="3">
         <v>3085097</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="3">
         <v>1345607</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="3">
         <v>2.2930000000000001</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="6">
         <v>185000</v>
       </c>
-      <c r="F19" s="4">
+      <c r="F19" s="5">
         <v>7.0999999999999995E-3</v>
       </c>
-      <c r="G19" s="3">
+      <c r="G19" s="4">
         <v>1699.1476824066201</v>
       </c>
       <c r="H19" s="3">
+        <v>20.440732199999999</v>
+      </c>
+      <c r="I19" s="4">
         <v>23.998244399999997</v>
       </c>
-      <c r="I19" s="6">
+      <c r="J19" s="2">
         <v>360000</v>
       </c>
-      <c r="J19" s="6">
+      <c r="K19" s="2">
         <v>130000</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="3">
         <v>2020</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="3">
         <v>2848472</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="3">
         <v>1350538</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="3">
         <v>2.109</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="6">
         <v>400000</v>
       </c>
-      <c r="F20" s="4">
+      <c r="F20" s="5">
         <v>4.1799999999999997E-2</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="4">
         <v>2802.37597291058</v>
       </c>
       <c r="H20" s="3">
+        <v>22.693819599999998</v>
+      </c>
+      <c r="I20" s="4">
         <v>25.689845599999998</v>
       </c>
-      <c r="I20" s="6">
+      <c r="J20" s="2">
         <v>700000</v>
       </c>
-      <c r="J20" s="6">
+      <c r="K20" s="2">
         <v>200000</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="3">
         <v>2021</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="3">
         <v>1951806</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="3">
         <v>1567262</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="3">
         <v>1.2450000000000001</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="6">
         <v>900000</v>
       </c>
-      <c r="F21" s="4">
+      <c r="F21" s="5">
         <v>0.30570000000000003</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" s="4">
         <v>6120.3674956709601</v>
       </c>
       <c r="H21" s="3">
+        <v>21.6579239</v>
+      </c>
+      <c r="I21" s="4">
         <v>25.333728399999998</v>
       </c>
-      <c r="I21" s="6">
+      <c r="J21" s="2">
         <v>2500000</v>
       </c>
-      <c r="J21" s="6">
+      <c r="K21" s="2">
         <v>200000</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
         <v>2022</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="3">
         <v>1551605</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="3">
         <v>1184237</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="3">
         <v>1.31</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="6">
         <v>2000000</v>
       </c>
-      <c r="F22" s="4">
+      <c r="F22" s="5">
         <v>0.38420000000000004</v>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" s="4">
         <v>12692.121336549801</v>
       </c>
       <c r="H22" s="3">
+        <v>19.9404842</v>
+      </c>
+      <c r="I22" s="4">
         <v>24.245223899999999</v>
       </c>
-      <c r="I22" s="6">
+      <c r="J22" s="2">
         <v>4000000</v>
       </c>
-      <c r="J22" s="6">
+      <c r="K22" s="2">
         <v>1800000</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
         <v>2023</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="3">
         <v>3080351</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="3">
         <v>1335667</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="3">
         <v>2.306</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="6">
         <v>2800000</v>
       </c>
-      <c r="F23" s="4">
+      <c r="F23" s="5">
         <v>9.0500000000000011E-2</v>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" s="4">
         <f xml:space="preserve"> G22*1.93</f>
         <v>24495.794179541113</v>
       </c>
       <c r="H23" s="3">
+        <v>19.949928099999997</v>
+      </c>
+      <c r="I23" s="4">
         <v>24.2511221</v>
       </c>
-      <c r="I23" s="6">
+      <c r="J23" s="2">
         <v>10000000</v>
       </c>
-      <c r="J23" s="6">
+      <c r="K23" s="2">
         <v>2200000</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="F30"/>
     </row>
   </sheetData>

</xml_diff>